<commit_message>
New benchmark results after bug fix - better now but still not perfect im afraid
</commit_message>
<xml_diff>
--- a/denoiser/benchmark/comparison_tables.xlsx
+++ b/denoiser/benchmark/comparison_tables.xlsx
@@ -12,7 +12,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="XUWgydfQIYmLjMF69nHIdnLaPgrHu5QrpSD4iaTnC9M="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="pNqs7JnhcYynYgNzUN2aHgAkj3Cu5bGDLLulCVHYQAA="/>
     </ext>
   </extLst>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="45">
   <si>
-    <t>PSNR Comparison (dB) — FastDVDNet vs VRT vs UNet</t>
+    <t>PSNR Comparison (dB)</t>
   </si>
   <si>
     <t>Noise Range (σ)</t>
@@ -93,7 +93,7 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>2026-02-22T15:31:56.723817</t>
+    <t>2026-03-01T12:34:21.337505</t>
   </si>
   <si>
     <t>Test videos:</t>
@@ -524,16 +524,16 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>21.42</v>
+        <v>21.4</v>
       </c>
       <c r="C4" s="4">
-        <v>26.5</v>
+        <v>32.93</v>
       </c>
       <c r="D4" s="5">
         <v>38.2</v>
       </c>
       <c r="E4" s="4">
-        <v>27.29</v>
+        <v>30.27</v>
       </c>
     </row>
     <row r="5">
@@ -541,16 +541,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>17.43</v>
+        <v>17.41</v>
       </c>
       <c r="C5" s="4">
-        <v>25.31</v>
+        <v>30.09</v>
       </c>
       <c r="D5" s="5">
         <v>33.31</v>
       </c>
       <c r="E5" s="4">
-        <v>26.86</v>
+        <v>28.28</v>
       </c>
     </row>
     <row r="6">
@@ -558,16 +558,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>14.06</v>
+        <v>14.04</v>
       </c>
       <c r="C6" s="4">
-        <v>23.61</v>
+        <v>26.72</v>
       </c>
       <c r="D6" s="5">
         <v>31.11</v>
       </c>
       <c r="E6" s="4">
-        <v>25.56</v>
+        <v>26.45</v>
       </c>
     </row>
     <row r="7">
@@ -575,16 +575,16 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>12.13</v>
+        <v>12.12</v>
       </c>
       <c r="C7" s="4">
-        <v>22.04</v>
+        <v>24.06</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="5">
-        <v>23.92</v>
+        <v>25.33</v>
       </c>
     </row>
     <row r="8">
@@ -592,16 +592,16 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>11.2</v>
+        <v>11.18</v>
       </c>
       <c r="C8" s="4">
-        <v>21.01</v>
+        <v>22.6</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="5">
-        <v>22.79</v>
+        <v>24.74</v>
       </c>
     </row>
     <row r="9">
@@ -609,16 +609,16 @@
         <v>12</v>
       </c>
       <c r="B9" s="4">
-        <v>9.72</v>
+        <v>9.71</v>
       </c>
       <c r="C9" s="4">
-        <v>19.01</v>
+        <v>19.88</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="5">
-        <v>20.6</v>
+        <v>23.64</v>
       </c>
     </row>
     <row r="10">
@@ -629,13 +629,13 @@
         <v>8.79</v>
       </c>
       <c r="C10" s="4">
-        <v>17.53</v>
+        <v>17.98</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="5">
-        <v>18.98</v>
+        <v>22.75</v>
       </c>
     </row>
     <row r="11">
@@ -646,13 +646,13 @@
         <v>8.52</v>
       </c>
       <c r="C11" s="4">
-        <v>17.07</v>
+        <v>17.4</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E11" s="5">
-        <v>18.51</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="12">
@@ -660,16 +660,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>7.89</v>
+        <v>7.9</v>
       </c>
       <c r="C12" s="4">
-        <v>15.92</v>
+        <v>16.02</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E12" s="5">
-        <v>17.34</v>
+        <v>21.66</v>
       </c>
     </row>
     <row r="13">
@@ -680,13 +680,13 @@
         <v>7.49</v>
       </c>
       <c r="C13" s="4">
-        <v>15.05</v>
+        <v>14.99</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="5">
-        <v>16.57</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="14">
@@ -694,16 +694,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>7.37</v>
+        <v>7.38</v>
       </c>
       <c r="C14" s="4">
-        <v>14.82</v>
+        <v>14.67</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="5">
-        <v>16.32</v>
+        <v>20.76</v>
       </c>
     </row>
     <row r="15">
@@ -714,13 +714,13 @@
         <v>7.13</v>
       </c>
       <c r="C15" s="4">
-        <v>14.34</v>
+        <v>13.99</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="5">
-        <v>15.85</v>
+        <v>20.25</v>
       </c>
     </row>
     <row r="16">
@@ -728,16 +728,16 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
-        <v>6.94</v>
+        <v>6.95</v>
       </c>
       <c r="C16" s="4">
-        <v>13.96</v>
+        <v>13.44</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="5">
-        <v>15.5</v>
+        <v>19.82</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1769,16 +1769,16 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>0.2297</v>
+        <v>0.4475</v>
       </c>
       <c r="C4" s="4">
-        <v>0.8146</v>
+        <v>0.9381</v>
       </c>
       <c r="D4" s="5">
         <v>0.9669</v>
       </c>
       <c r="E4" s="4">
-        <v>0.8348</v>
+        <v>0.8883</v>
       </c>
     </row>
     <row r="5">
@@ -1786,16 +1786,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>0.1283</v>
+        <v>0.3084</v>
       </c>
       <c r="C5" s="4">
-        <v>0.7952</v>
+        <v>0.901</v>
       </c>
       <c r="D5" s="5">
         <v>0.9175</v>
       </c>
       <c r="E5" s="4">
-        <v>0.8279</v>
+        <v>0.841</v>
       </c>
     </row>
     <row r="6">
@@ -1803,16 +1803,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>0.0727</v>
+        <v>0.2035</v>
       </c>
       <c r="C6" s="4">
-        <v>0.7673</v>
+        <v>0.8395</v>
       </c>
       <c r="D6" s="5">
         <v>0.88</v>
       </c>
       <c r="E6" s="4">
-        <v>0.8139</v>
+        <v>0.7807</v>
       </c>
     </row>
     <row r="7">
@@ -1820,16 +1820,16 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>0.0501</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0.7276</v>
+        <v>0.1503</v>
+      </c>
+      <c r="C7" s="5">
+        <v>0.7739</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="5">
-        <v>0.7988</v>
+      <c r="E7" s="4">
+        <v>0.7306</v>
       </c>
     </row>
     <row r="8">
@@ -1837,16 +1837,16 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>0.041</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0.685</v>
+        <v>0.1264</v>
+      </c>
+      <c r="C8" s="5">
+        <v>0.7154</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="5">
-        <v>0.7883</v>
+      <c r="E8" s="4">
+        <v>0.6998</v>
       </c>
     </row>
     <row r="9">
@@ -1854,16 +1854,16 @@
         <v>12</v>
       </c>
       <c r="B9" s="4">
-        <v>0.0289</v>
+        <v>0.0918</v>
       </c>
       <c r="C9" s="4">
-        <v>0.643</v>
+        <v>0.5365</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="5">
-        <v>0.7656</v>
+        <v>0.6416</v>
       </c>
     </row>
     <row r="10">
@@ -1871,16 +1871,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="4">
-        <v>0.0224</v>
+        <v>0.0715</v>
       </c>
       <c r="C10" s="4">
-        <v>0.5768</v>
+        <v>0.373</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="5">
-        <v>0.7462</v>
+        <v>0.5932</v>
       </c>
     </row>
     <row r="11">
@@ -1888,16 +1888,16 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>0.0207</v>
+        <v>0.0661</v>
       </c>
       <c r="C11" s="4">
-        <v>0.5554</v>
+        <v>0.3268</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E11" s="5">
-        <v>0.7399</v>
+        <v>0.5775</v>
       </c>
     </row>
     <row r="12">
@@ -1905,16 +1905,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>0.0169</v>
+        <v>0.0535</v>
       </c>
       <c r="C12" s="4">
-        <v>0.522</v>
+        <v>0.2395</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E12" s="5">
-        <v>0.723</v>
+        <v>0.5334</v>
       </c>
     </row>
     <row r="13">
@@ -1922,16 +1922,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="4">
-        <v>0.0147</v>
+        <v>0.0458</v>
       </c>
       <c r="C13" s="4">
-        <v>0.4763</v>
+        <v>0.1844</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="5">
-        <v>0.7108</v>
+        <v>0.5022</v>
       </c>
     </row>
     <row r="14">
@@ -1939,16 +1939,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>0.014</v>
+        <v>0.0434</v>
       </c>
       <c r="C14" s="4">
-        <v>0.4642</v>
+        <v>0.1671</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="5">
-        <v>0.7068</v>
+        <v>0.4892</v>
       </c>
     </row>
     <row r="15">
@@ -1956,16 +1956,16 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>0.0127</v>
+        <v>0.0389</v>
       </c>
       <c r="C15" s="4">
-        <v>0.4151</v>
+        <v>0.1371</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="5">
-        <v>0.6985</v>
+        <v>0.4656</v>
       </c>
     </row>
     <row r="16">
@@ -1973,16 +1973,16 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
-        <v>0.0118</v>
+        <v>0.0358</v>
       </c>
       <c r="C16" s="4">
-        <v>0.3803</v>
+        <v>0.1183</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="5">
-        <v>0.6921</v>
+        <v>0.446</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3011,13 +3011,13 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>5.08</v>
+        <v>11.53</v>
       </c>
       <c r="C4" s="5">
-        <v>16.78</v>
+        <v>16.8</v>
       </c>
       <c r="D4" s="4">
-        <v>5.87</v>
+        <v>8.86</v>
       </c>
     </row>
     <row r="5">
@@ -3025,13 +3025,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>7.88</v>
+        <v>12.68</v>
       </c>
       <c r="C5" s="5">
-        <v>15.88</v>
+        <v>15.9</v>
       </c>
       <c r="D5" s="4">
-        <v>9.42</v>
+        <v>10.87</v>
       </c>
     </row>
     <row r="6">
@@ -3039,13 +3039,13 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>9.55</v>
+        <v>12.67</v>
       </c>
       <c r="C6" s="5">
-        <v>17.05</v>
+        <v>17.07</v>
       </c>
       <c r="D6" s="4">
-        <v>11.5</v>
+        <v>12.41</v>
       </c>
     </row>
     <row r="7">
@@ -3053,13 +3053,13 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>9.91</v>
+        <v>11.95</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="5">
-        <v>11.79</v>
+        <v>13.22</v>
       </c>
     </row>
     <row r="8">
@@ -3067,13 +3067,13 @@
         <v>11</v>
       </c>
       <c r="B8" s="4">
-        <v>9.81</v>
+        <v>11.41</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="5">
-        <v>11.6</v>
+        <v>13.56</v>
       </c>
     </row>
     <row r="9">
@@ -3081,13 +3081,13 @@
         <v>12</v>
       </c>
       <c r="B9" s="4">
-        <v>9.29</v>
+        <v>10.17</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="5">
-        <v>10.88</v>
+        <v>13.93</v>
       </c>
     </row>
     <row r="10">
@@ -3095,13 +3095,13 @@
         <v>13</v>
       </c>
       <c r="B10" s="4">
-        <v>8.75</v>
+        <v>9.19</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="5">
-        <v>10.2</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="11">
@@ -3109,13 +3109,13 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>8.55</v>
+        <v>8.88</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="5">
-        <v>9.99</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="12">
@@ -3123,13 +3123,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>8.03</v>
+        <v>8.12</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="5">
-        <v>9.44</v>
+        <v>13.76</v>
       </c>
     </row>
     <row r="13">
@@ -3137,13 +3137,13 @@
         <v>16</v>
       </c>
       <c r="B13" s="4">
-        <v>7.56</v>
+        <v>7.5</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="5">
-        <v>9.07</v>
+        <v>13.51</v>
       </c>
     </row>
     <row r="14">
@@ -3151,13 +3151,13 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>7.46</v>
+        <v>7.29</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="5">
-        <v>8.96</v>
+        <v>13.39</v>
       </c>
     </row>
     <row r="15">
@@ -3165,13 +3165,13 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>7.22</v>
+        <v>6.85</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="5">
-        <v>8.73</v>
+        <v>13.12</v>
       </c>
     </row>
     <row r="16">
@@ -3179,13 +3179,13 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
-        <v>7.02</v>
+        <v>6.49</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="5">
-        <v>8.55</v>
+        <v>12.87</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Fix bug in benchmark
</commit_message>
<xml_diff>
--- a/denoiser/benchmark/comparison_tables.xlsx
+++ b/denoiser/benchmark/comparison_tables.xlsx
@@ -12,14 +12,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="pNqs7JnhcYynYgNzUN2aHgAkj3Cu5bGDLLulCVHYQAA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="MJkLJZEbEIGq6bWIOgUM8Yph2wzYeDKQ1UdZRAINTcc="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="47">
   <si>
     <t>PSNR Comparison (dB)</t>
   </si>
@@ -39,13 +39,19 @@
     <t>YourUNet</t>
   </si>
   <si>
-    <t>5-25</t>
+    <t>σ=10</t>
   </si>
   <si>
-    <t>25-45</t>
+    <t>σ=20</t>
   </si>
   <si>
-    <t>45-65</t>
+    <t>σ=30</t>
+  </si>
+  <si>
+    <t>σ=40</t>
+  </si>
+  <si>
+    <t>σ=50</t>
   </si>
   <si>
     <t>65-85</t>
@@ -93,7 +99,7 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>2026-03-01T12:34:21.337505</t>
+    <t>2026-03-01T13:57:39.048414</t>
   </si>
   <si>
     <t>Test videos:</t>
@@ -524,16 +530,16 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>21.4</v>
+        <v>28.2</v>
       </c>
       <c r="C4" s="4">
-        <v>32.93</v>
+        <v>36.66</v>
       </c>
       <c r="D4" s="5">
-        <v>38.2</v>
+        <v>40.82</v>
       </c>
       <c r="E4" s="4">
-        <v>30.27</v>
+        <v>33.03</v>
       </c>
     </row>
     <row r="5">
@@ -541,16 +547,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>17.41</v>
+        <v>22.32</v>
       </c>
       <c r="C5" s="4">
-        <v>30.09</v>
+        <v>33.48</v>
       </c>
       <c r="D5" s="5">
-        <v>33.31</v>
+        <v>38.15</v>
       </c>
       <c r="E5" s="4">
-        <v>28.28</v>
+        <v>30.69</v>
       </c>
     </row>
     <row r="6">
@@ -558,16 +564,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>14.04</v>
+        <v>18.98</v>
       </c>
       <c r="C6" s="4">
-        <v>26.72</v>
+        <v>31.3</v>
       </c>
       <c r="D6" s="5">
-        <v>31.11</v>
+        <v>36.52</v>
       </c>
       <c r="E6" s="4">
-        <v>26.45</v>
+        <v>29.08</v>
       </c>
     </row>
     <row r="7">
@@ -575,50 +581,50 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>12.12</v>
+        <v>16.7</v>
       </c>
       <c r="C7" s="4">
-        <v>24.06</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="5">
-        <v>25.33</v>
+        <v>29.49</v>
+      </c>
+      <c r="D7" s="5">
+        <v>35.32</v>
+      </c>
+      <c r="E7" s="4">
+        <v>27.91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4">
-        <v>11.18</v>
+        <v>15.0</v>
       </c>
       <c r="C8" s="4">
-        <v>22.6</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="5">
-        <v>24.74</v>
+        <v>27.82</v>
+      </c>
+      <c r="D8" s="5">
+        <v>34.36</v>
+      </c>
+      <c r="E8" s="4">
+        <v>26.99</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4">
+        <v>12.12</v>
+      </c>
+      <c r="C9" s="4">
+        <v>24.06</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4">
-        <v>9.71</v>
-      </c>
-      <c r="C9" s="4">
-        <v>19.88</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>10</v>
-      </c>
       <c r="E9" s="5">
-        <v>23.64</v>
+        <v>25.33</v>
       </c>
     </row>
     <row r="10">
@@ -626,16 +632,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="4">
-        <v>8.79</v>
+        <v>11.18</v>
       </c>
       <c r="C10" s="4">
-        <v>17.98</v>
+        <v>22.6</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5">
-        <v>22.75</v>
+        <v>24.74</v>
       </c>
     </row>
     <row r="11">
@@ -643,16 +649,16 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>8.52</v>
+        <v>9.71</v>
       </c>
       <c r="C11" s="4">
-        <v>17.4</v>
+        <v>19.88</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E11" s="5">
-        <v>22.5</v>
+        <v>23.64</v>
       </c>
     </row>
     <row r="12">
@@ -660,16 +666,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>7.9</v>
+        <v>8.79</v>
       </c>
       <c r="C12" s="4">
-        <v>16.02</v>
+        <v>17.98</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="5">
-        <v>21.66</v>
+        <v>22.75</v>
       </c>
     </row>
     <row r="13">
@@ -677,16 +683,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="4">
-        <v>7.49</v>
+        <v>8.52</v>
       </c>
       <c r="C13" s="4">
-        <v>14.99</v>
+        <v>17.4</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E13" s="5">
-        <v>21.0</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="14">
@@ -694,16 +700,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>7.38</v>
+        <v>7.9</v>
       </c>
       <c r="C14" s="4">
-        <v>14.67</v>
+        <v>16.02</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E14" s="5">
-        <v>20.76</v>
+        <v>21.66</v>
       </c>
     </row>
     <row r="15">
@@ -711,16 +717,16 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>7.13</v>
+        <v>7.49</v>
       </c>
       <c r="C15" s="4">
-        <v>13.99</v>
+        <v>14.99</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E15" s="5">
-        <v>20.25</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="16">
@@ -728,15 +734,49 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
+        <v>7.38</v>
+      </c>
+      <c r="C16" s="4">
+        <v>14.67</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="5">
+        <v>20.76</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4">
+        <v>7.13</v>
+      </c>
+      <c r="C17" s="4">
+        <v>13.99</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="5">
+        <v>20.25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4">
         <v>6.95</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C18" s="4">
         <v>13.44</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="5">
+      <c r="D18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="5">
         <v>19.82</v>
       </c>
     </row>
@@ -1744,7 +1784,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -1769,16 +1809,16 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>0.4475</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0.9381</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0.9669</v>
+        <v>0.7026</v>
+      </c>
+      <c r="C4" s="5">
+        <v>0.9692</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="E4" s="4">
-        <v>0.8883</v>
+        <v>0.9368</v>
       </c>
     </row>
     <row r="5">
@@ -1786,16 +1826,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>0.3084</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0.901</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0.9175</v>
+        <v>0.4814</v>
+      </c>
+      <c r="C5" s="5">
+        <v>0.944</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="E5" s="4">
-        <v>0.841</v>
+        <v>0.8969</v>
       </c>
     </row>
     <row r="6">
@@ -1803,16 +1843,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>0.2035</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.8395</v>
-      </c>
-      <c r="D6" s="5">
-        <v>0.88</v>
+        <v>0.3614</v>
+      </c>
+      <c r="C6" s="5">
+        <v>0.9183</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="E6" s="4">
-        <v>0.7807</v>
+        <v>0.8615</v>
       </c>
     </row>
     <row r="7">
@@ -1820,50 +1860,50 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>0.1503</v>
+        <v>0.2856</v>
       </c>
       <c r="C7" s="5">
-        <v>0.7739</v>
+        <v>0.8916</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E7" s="4">
-        <v>0.7306</v>
+        <v>0.8308</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4">
-        <v>0.1264</v>
+        <v>0.2319</v>
       </c>
       <c r="C8" s="5">
-        <v>0.7154</v>
+        <v>0.8627</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" s="4">
-        <v>0.6998</v>
+        <v>0.8009</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.1503</v>
+      </c>
+      <c r="C9" s="5">
+        <v>0.7739</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4">
-        <v>0.0918</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0.5365</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0.6416</v>
+      <c r="E9" s="4">
+        <v>0.7306</v>
       </c>
     </row>
     <row r="10">
@@ -1871,16 +1911,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="4">
-        <v>0.0715</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0.373</v>
+        <v>0.1264</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.7154</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0.5932</v>
+        <v>12</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0.6998</v>
       </c>
     </row>
     <row r="11">
@@ -1888,16 +1928,16 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>0.0661</v>
+        <v>0.0918</v>
       </c>
       <c r="C11" s="4">
-        <v>0.3268</v>
+        <v>0.5365</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E11" s="5">
-        <v>0.5775</v>
+        <v>0.6416</v>
       </c>
     </row>
     <row r="12">
@@ -1905,16 +1945,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>0.0535</v>
+        <v>0.0715</v>
       </c>
       <c r="C12" s="4">
-        <v>0.2395</v>
+        <v>0.373</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="5">
-        <v>0.5334</v>
+        <v>0.5932</v>
       </c>
     </row>
     <row r="13">
@@ -1922,16 +1962,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="4">
-        <v>0.0458</v>
+        <v>0.0661</v>
       </c>
       <c r="C13" s="4">
-        <v>0.1844</v>
+        <v>0.3268</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E13" s="5">
-        <v>0.5022</v>
+        <v>0.5775</v>
       </c>
     </row>
     <row r="14">
@@ -1939,16 +1979,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>0.0434</v>
+        <v>0.0535</v>
       </c>
       <c r="C14" s="4">
-        <v>0.1671</v>
+        <v>0.2395</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E14" s="5">
-        <v>0.4892</v>
+        <v>0.5334</v>
       </c>
     </row>
     <row r="15">
@@ -1956,16 +1996,16 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>0.0389</v>
+        <v>0.0458</v>
       </c>
       <c r="C15" s="4">
-        <v>0.1371</v>
+        <v>0.1844</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E15" s="5">
-        <v>0.4656</v>
+        <v>0.5022</v>
       </c>
     </row>
     <row r="16">
@@ -1973,15 +2013,49 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
+        <v>0.0434</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0.1671</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0.4892</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.0389</v>
+      </c>
+      <c r="C17" s="4">
+        <v>0.1371</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0.4656</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4">
         <v>0.0358</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C18" s="4">
         <v>0.1183</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="5">
+      <c r="D18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="5">
         <v>0.446</v>
       </c>
     </row>
@@ -2989,7 +3063,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -3011,13 +3085,13 @@
         <v>6</v>
       </c>
       <c r="B4" s="4">
-        <v>11.53</v>
+        <v>8.46</v>
       </c>
       <c r="C4" s="5">
-        <v>16.8</v>
+        <v>12.62</v>
       </c>
       <c r="D4" s="4">
-        <v>8.86</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="5">
@@ -3025,13 +3099,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="4">
-        <v>12.68</v>
+        <v>11.16</v>
       </c>
       <c r="C5" s="5">
-        <v>15.9</v>
+        <v>15.83</v>
       </c>
       <c r="D5" s="4">
-        <v>10.87</v>
+        <v>8.37</v>
       </c>
     </row>
     <row r="6">
@@ -3039,13 +3113,13 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>12.67</v>
+        <v>12.32</v>
       </c>
       <c r="C6" s="5">
-        <v>17.07</v>
+        <v>17.54</v>
       </c>
       <c r="D6" s="4">
-        <v>12.41</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="7">
@@ -3053,41 +3127,41 @@
         <v>9</v>
       </c>
       <c r="B7" s="4">
-        <v>11.95</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="5">
-        <v>13.22</v>
+        <v>12.79</v>
+      </c>
+      <c r="C7" s="5">
+        <v>18.62</v>
+      </c>
+      <c r="D7" s="4">
+        <v>11.21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4">
-        <v>11.41</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="5">
-        <v>13.56</v>
+        <v>12.83</v>
+      </c>
+      <c r="C8" s="5">
+        <v>19.36</v>
+      </c>
+      <c r="D8" s="4">
+        <v>11.99</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4">
+        <v>11.95</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4">
-        <v>10.17</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>10</v>
-      </c>
       <c r="D9" s="5">
-        <v>13.93</v>
+        <v>13.22</v>
       </c>
     </row>
     <row r="10">
@@ -3095,13 +3169,13 @@
         <v>13</v>
       </c>
       <c r="B10" s="4">
-        <v>9.19</v>
+        <v>11.41</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D10" s="5">
-        <v>13.97</v>
+        <v>13.56</v>
       </c>
     </row>
     <row r="11">
@@ -3109,13 +3183,13 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>8.88</v>
+        <v>10.17</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D11" s="5">
-        <v>13.97</v>
+        <v>13.93</v>
       </c>
     </row>
     <row r="12">
@@ -3123,13 +3197,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="4">
-        <v>8.12</v>
+        <v>9.19</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" s="5">
-        <v>13.76</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="13">
@@ -3137,13 +3211,13 @@
         <v>16</v>
       </c>
       <c r="B13" s="4">
-        <v>7.5</v>
+        <v>8.88</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="5">
-        <v>13.51</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="14">
@@ -3151,13 +3225,13 @@
         <v>17</v>
       </c>
       <c r="B14" s="4">
-        <v>7.29</v>
+        <v>8.12</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D14" s="5">
-        <v>13.39</v>
+        <v>13.76</v>
       </c>
     </row>
     <row r="15">
@@ -3165,13 +3239,13 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>6.85</v>
+        <v>7.5</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" s="5">
-        <v>13.12</v>
+        <v>13.51</v>
       </c>
     </row>
     <row r="16">
@@ -3179,12 +3253,40 @@
         <v>19</v>
       </c>
       <c r="B16" s="4">
+        <v>7.29</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="5">
+        <v>13.39</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4">
+        <v>6.85</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="5">
+        <v>13.12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4">
         <v>6.49</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="5">
+      <c r="C18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="5">
         <v>12.87</v>
       </c>
     </row>
@@ -4193,7 +4295,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
@@ -4201,42 +4303,42 @@
     </row>
     <row r="3">
       <c r="A3" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
@@ -4244,31 +4346,31 @@
     </row>
     <row r="9">
       <c r="A9" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13">
@@ -4276,7 +4378,7 @@
     </row>
     <row r="14">
       <c r="A14" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -4284,7 +4386,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16">
@@ -4292,7 +4394,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -4300,7 +4402,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -4308,7 +4410,7 @@
     </row>
     <row r="19">
       <c r="A19" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>